<commit_message>
research: second pass (glamping, equestrian, fee norms) and docs/RESEARCH.md with generated coverage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-output/01-garden-multifamily/estimate.xlsx
+++ b/docs/sample-output/01-garden-multifamily/estimate.xlsx
@@ -16,12 +16,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="372">
   <si>
     <t>FINISHES SOLUTIONS</t>
   </si>
   <si>
-    <t>Total Project Cost — Summary   ·   Cedar Hollow — garden multifamily · Total $66,654,800</t>
+    <t>Total Project Cost — Summary   ·   Cedar Hollow — garden multifamily · Total $66,218,599</t>
   </si>
   <si>
     <t>COST SUMMARY</t>
@@ -90,7 +90,7 @@
     <t>Research data version</t>
   </si>
   <si>
-    <t>2026.7c60a42879</t>
+    <t>2026.0c737c8255</t>
   </si>
   <si>
     <t>Engine</t>
@@ -99,10 +99,10 @@
     <t>budget-engine-2.0.0</t>
   </si>
   <si>
-    <t>All defaults come from the research data shipped with the app (2026.7c60a42879), escalated to the construction midpoint and adjusted to the project location. Values marked "Derived estimate — verify" have no direct published source.</t>
-  </si>
-  <si>
-    <t>Cost by Component   ·   Cedar Hollow — garden multifamily · Total $66,654,800</t>
+    <t>All defaults come from the research data shipped with the app (2026.0c737c8255), escalated to the construction midpoint and adjusted to the project location. Values marked "Derived estimate — verify" have no direct published source.</t>
+  </si>
+  <si>
+    <t>Cost by Component   ·   Cedar Hollow — garden multifamily · Total $66,218,599</t>
   </si>
   <si>
     <t>Component</t>
@@ -147,7 +147,7 @@
     <t>within ($150,000–$420,000)</t>
   </si>
   <si>
-    <t>Cost by Phase   ·   Cedar Hollow — garden multifamily · Total $66,654,800</t>
+    <t>Cost by Phase   ·   Cedar Hollow — garden multifamily · Total $66,218,599</t>
   </si>
   <si>
     <t>Phase</t>
@@ -189,7 +189,7 @@
     <t>7.3%</t>
   </si>
   <si>
-    <t>Line-Item Detail   ·   Cedar Hollow — garden multifamily · Total $66,654,800</t>
+    <t>Line-Item Detail   ·   Cedar Hollow — garden multifamily · Total $66,218,599</t>
   </si>
   <si>
     <t>Group</t>
@@ -477,7 +477,7 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Draw Schedules   ·   Cedar Hollow — garden multifamily · Total $66,654,800</t>
+    <t>Draw Schedules   ·   Cedar Hollow — garden multifamily · Total $66,218,599</t>
   </si>
   <si>
     <t>PHASE 1 — MONTHLY DRAWS</t>
@@ -567,7 +567,7 @@
     <t>2029-04</t>
   </si>
   <si>
-    <t>Sources &amp; Assumptions   ·   Cedar Hollow — garden multifamily · Total $66,654,800</t>
+    <t>Sources &amp; Assumptions   ·   Cedar Hollow — garden multifamily · Total $66,218,599</t>
   </si>
   <si>
     <t>ASSUMPTIONS</t>
@@ -603,7 +603,7 @@
     <t>LTC 60%, rate 7.00%, fee 1.00%</t>
   </si>
   <si>
-    <t>SOURCES (45)</t>
+    <t>SOURCES (46)</t>
   </si>
   <si>
     <t>Ref</t>
@@ -1117,6 +1117,21 @@
   </si>
   <si>
     <t>109.12 USD/nrsf (2019)</t>
+  </si>
+  <si>
+    <t>residential/single-family.json#e10</t>
+  </si>
+  <si>
+    <t>Cost of Constructing a Home-2024 (Special Study for Housing Economics)</t>
+  </si>
+  <si>
+    <t>National Association of Home Builders (Eric Lynch)</t>
+  </si>
+  <si>
+    <t>26747 USD/unit (2024)</t>
+  </si>
+  <si>
+    <t>https://nahb.org/-/media/AB4EFC742624475A97A0A62189986FF8.ashx</t>
   </si>
 </sst>
 </file>
@@ -1714,7 +1729,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="5">
-        <v>3247841.28</v>
+        <v>2871111.36</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1722,7 +1737,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="5">
-        <v>2276603.59</v>
+        <v>2260780.93</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -1730,7 +1745,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="5">
-        <v>2534307.05</v>
+        <v>2509494.91</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -1738,7 +1753,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="5">
-        <v>517683.01</v>
+        <v>498846.52</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -1746,7 +1761,7 @@
         <v>12</v>
       </c>
       <c r="B14" s="7">
-        <v>15792253.89</v>
+        <v>15356052.68</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1762,7 +1777,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="7">
-        <v>66654800.31</v>
+        <v>66218599.1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1801,7 +1816,7 @@
         <v>22</v>
       </c>
       <c r="B21" s="5">
-        <v>6110023.361750001</v>
+        <v>6070038.2508333335</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -1929,19 +1944,19 @@
         <v>45933746.42</v>
       </c>
       <c r="E5" s="13">
-        <v>15792253.89</v>
+        <v>15356052.68</v>
       </c>
       <c r="F5" s="13">
         <v>4928800</v>
       </c>
       <c r="G5" s="13">
-        <v>66654800.31</v>
+        <v>66218599.1</v>
       </c>
       <c r="H5" s="13">
-        <v>277728.334625</v>
+        <v>275910.82958333334</v>
       </c>
       <c r="I5" s="14">
-        <v>264.50317583333333</v>
+        <v>262.77221865079366</v>
       </c>
       <c r="J5" s="12" t="s">
         <v>42</v>
@@ -1957,13 +1972,13 @@
         <v>45933746.42</v>
       </c>
       <c r="E6" s="16">
-        <v>15792253.89</v>
+        <v>15356052.68</v>
       </c>
       <c r="F6" s="16">
         <v>4928800</v>
       </c>
       <c r="G6" s="16">
-        <v>66654800.31</v>
+        <v>66218599.1</v>
       </c>
       <c r="H6" s="15"/>
       <c r="I6" s="15"/>
@@ -2079,19 +2094,19 @@
         <v>45933746.42</v>
       </c>
       <c r="G5" s="13">
-        <v>15792253.89</v>
+        <v>15356052.68</v>
       </c>
       <c r="H5" s="13">
         <v>4928800</v>
       </c>
       <c r="I5" s="13">
-        <v>66654800.31</v>
+        <v>66218599.1</v>
       </c>
       <c r="J5" s="13">
-        <v>39992880.19</v>
+        <v>39731159.46</v>
       </c>
       <c r="K5" s="13">
-        <v>2134378.25</v>
+        <v>2112183.32</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -2106,13 +2121,13 @@
         <v>45933746.42</v>
       </c>
       <c r="G6" s="16">
-        <v>15792253.89</v>
+        <v>15356052.68</v>
       </c>
       <c r="H6" s="16">
         <v>4928800</v>
       </c>
       <c r="I6" s="16">
-        <v>66654800.31</v>
+        <v>66218599.1</v>
       </c>
       <c r="J6" s="15"/>
       <c r="K6" s="15"/>
@@ -3341,10 +3356,10 @@
         <v>137</v>
       </c>
       <c r="H43" s="14">
-        <v>4838.18</v>
+        <v>3407.22</v>
       </c>
       <c r="I43" s="13">
-        <v>696697.92</v>
+        <v>490639.68</v>
       </c>
       <c r="J43" s="12" t="s">
         <v>69</v>
@@ -3373,10 +3388,10 @@
         <v>137</v>
       </c>
       <c r="H44" s="14">
-        <v>4592.44</v>
+        <v>3407.22</v>
       </c>
       <c r="I44" s="13">
-        <v>661311.36</v>
+        <v>490639.68</v>
       </c>
       <c r="J44" s="12" t="s">
         <v>69</v>
@@ -3406,7 +3421,7 @@
       </c>
       <c r="H45" s="18"/>
       <c r="I45" s="13">
-        <v>517683.01</v>
+        <v>498846.52</v>
       </c>
       <c r="J45" s="12" t="s">
         <v>69</v>
@@ -3552,7 +3567,7 @@
       </c>
       <c r="H50" s="18"/>
       <c r="I50" s="13">
-        <v>2276603.59</v>
+        <v>2260780.93</v>
       </c>
       <c r="J50" s="12" t="s">
         <v>69</v>
@@ -3580,7 +3595,7 @@
       </c>
       <c r="H51" s="18"/>
       <c r="I51" s="13">
-        <v>2134378.25</v>
+        <v>2112183.32</v>
       </c>
       <c r="J51" s="12" t="s">
         <v>69</v>
@@ -3608,7 +3623,7 @@
       </c>
       <c r="H52" s="18"/>
       <c r="I52" s="13">
-        <v>399928.8</v>
+        <v>397311.59</v>
       </c>
       <c r="J52" s="12" t="s">
         <v>69</v>
@@ -3628,7 +3643,7 @@
       <c r="G53" s="15"/>
       <c r="H53" s="15"/>
       <c r="I53" s="16">
-        <v>66654800.31</v>
+        <v>66218599.1</v>
       </c>
       <c r="J53" s="15"/>
     </row>
@@ -3727,13 +3742,13 @@
         <v>0</v>
       </c>
       <c r="C6" s="13">
-        <v>7392631.41</v>
+        <v>7015901.49</v>
       </c>
       <c r="D6" s="13">
         <v>4928800</v>
       </c>
       <c r="E6" s="13">
-        <v>12721360.21</v>
+        <v>12342013.08</v>
       </c>
       <c r="F6" s="13">
         <v>0</v>
@@ -3753,13 +3768,13 @@
         <v>181100.67</v>
       </c>
       <c r="C7" s="13">
-        <v>234612.6</v>
+        <v>233226.24</v>
       </c>
       <c r="D7" s="13">
         <v>0</v>
       </c>
       <c r="E7" s="13">
-        <v>415713.27</v>
+        <v>414326.91</v>
       </c>
       <c r="F7" s="13">
         <v>0</v>
@@ -3779,13 +3794,13 @@
         <v>540445.9</v>
       </c>
       <c r="C8" s="13">
-        <v>234612.6</v>
+        <v>233226.24</v>
       </c>
       <c r="D8" s="13">
         <v>0</v>
       </c>
       <c r="E8" s="13">
-        <v>775058.5</v>
+        <v>773672.14</v>
       </c>
       <c r="F8" s="13">
         <v>0</v>
@@ -3805,13 +3820,13 @@
         <v>891267.95</v>
       </c>
       <c r="C9" s="13">
-        <v>234612.6</v>
+        <v>233226.24</v>
       </c>
       <c r="D9" s="13">
         <v>0</v>
       </c>
       <c r="E9" s="13">
-        <v>1125880.55</v>
+        <v>1124494.19</v>
       </c>
       <c r="F9" s="13">
         <v>0</v>
@@ -3831,13 +3846,13 @@
         <v>1228034.25</v>
       </c>
       <c r="C10" s="13">
-        <v>234612.62</v>
+        <v>233226.26</v>
       </c>
       <c r="D10" s="13">
         <v>0</v>
       </c>
       <c r="E10" s="13">
-        <v>1462646.87</v>
+        <v>1461260.51</v>
       </c>
       <c r="F10" s="13">
         <v>0</v>
@@ -3857,13 +3872,13 @@
         <v>1545433.69</v>
       </c>
       <c r="C11" s="13">
-        <v>234612.6</v>
+        <v>233226.24</v>
       </c>
       <c r="D11" s="13">
         <v>0</v>
       </c>
       <c r="E11" s="13">
-        <v>1780046.29</v>
+        <v>1778659.93</v>
       </c>
       <c r="F11" s="13">
         <v>0</v>
@@ -3883,13 +3898,13 @@
         <v>1838460.69</v>
       </c>
       <c r="C12" s="13">
-        <v>234612.6</v>
+        <v>233226.24</v>
       </c>
       <c r="D12" s="13">
         <v>0</v>
       </c>
       <c r="E12" s="13">
-        <v>2073073.29</v>
+        <v>2071686.93</v>
       </c>
       <c r="F12" s="13">
         <v>0</v>
@@ -3909,13 +3924,13 @@
         <v>2102494.1</v>
       </c>
       <c r="C13" s="13">
-        <v>234612.67</v>
+        <v>233226.3</v>
       </c>
       <c r="D13" s="13">
         <v>0</v>
       </c>
       <c r="E13" s="13">
-        <v>2337106.77</v>
+        <v>2335720.4</v>
       </c>
       <c r="F13" s="13">
         <v>0</v>
@@ -3935,13 +3950,13 @@
         <v>2333369.89</v>
       </c>
       <c r="C14" s="13">
-        <v>234612.6</v>
+        <v>233226.24</v>
       </c>
       <c r="D14" s="13">
         <v>0</v>
       </c>
       <c r="E14" s="13">
-        <v>2567982.49</v>
+        <v>2566596.13</v>
       </c>
       <c r="F14" s="13">
         <v>0</v>
@@ -3961,22 +3976,22 @@
         <v>2527447.05</v>
       </c>
       <c r="C15" s="13">
-        <v>234612.6</v>
+        <v>233226.23</v>
       </c>
       <c r="D15" s="13">
         <v>0</v>
       </c>
       <c r="E15" s="13">
-        <v>1403051.88</v>
+        <v>1619009.42</v>
       </c>
       <c r="F15" s="13">
-        <v>1359007.77</v>
+        <v>1141663.86</v>
       </c>
       <c r="G15" s="13">
         <v>0</v>
       </c>
       <c r="H15" s="13">
-        <v>1359007.77</v>
+        <v>1141663.86</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -3987,7 +4002,7 @@
         <v>2681664.9</v>
       </c>
       <c r="C16" s="13">
-        <v>234612.66</v>
+        <v>233226.3</v>
       </c>
       <c r="D16" s="13">
         <v>0</v>
@@ -3996,13 +4011,13 @@
         <v>0</v>
       </c>
       <c r="F16" s="13">
-        <v>2916277.56</v>
+        <v>2914891.2</v>
       </c>
       <c r="G16" s="13">
-        <v>7927.55</v>
+        <v>6659.71</v>
       </c>
       <c r="H16" s="13">
-        <v>4283212.88</v>
+        <v>4063214.77</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -4013,7 +4028,7 @@
         <v>2793591.23</v>
       </c>
       <c r="C17" s="13">
-        <v>234612.6</v>
+        <v>233226.23</v>
       </c>
       <c r="D17" s="13">
         <v>0</v>
@@ -4022,13 +4037,13 @@
         <v>0</v>
       </c>
       <c r="F17" s="13">
-        <v>3028203.83</v>
+        <v>3026817.46</v>
       </c>
       <c r="G17" s="13">
-        <v>24985.41</v>
+        <v>23702.09</v>
       </c>
       <c r="H17" s="13">
-        <v>7336402.12</v>
+        <v>7113734.32</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -4039,7 +4054,7 @@
         <v>2861460.98</v>
       </c>
       <c r="C18" s="13">
-        <v>234612.6</v>
+        <v>233226.23</v>
       </c>
       <c r="D18" s="13">
         <v>0</v>
@@ -4048,13 +4063,13 @@
         <v>0</v>
       </c>
       <c r="F18" s="13">
-        <v>3096073.58</v>
+        <v>3094687.21</v>
       </c>
       <c r="G18" s="13">
-        <v>42795.68</v>
+        <v>41496.78</v>
       </c>
       <c r="H18" s="13">
-        <v>10475271.38</v>
+        <v>10249918.31</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -4065,7 +4080,7 @@
         <v>2884203.81</v>
       </c>
       <c r="C19" s="13">
-        <v>234612.66</v>
+        <v>233226.29</v>
       </c>
       <c r="D19" s="13">
         <v>0</v>
@@ -4074,13 +4089,13 @@
         <v>0</v>
       </c>
       <c r="F19" s="13">
-        <v>3118816.47</v>
+        <v>3117430.1</v>
       </c>
       <c r="G19" s="13">
-        <v>61105.75</v>
+        <v>59791.19</v>
       </c>
       <c r="H19" s="13">
-        <v>13655193.6</v>
+        <v>13427139.6</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -4091,7 +4106,7 @@
         <v>2861461</v>
       </c>
       <c r="C20" s="13">
-        <v>234612.65</v>
+        <v>233226.28</v>
       </c>
       <c r="D20" s="13">
         <v>0</v>
@@ -4100,13 +4115,13 @@
         <v>0</v>
       </c>
       <c r="F20" s="13">
-        <v>3096073.65</v>
+        <v>3094687.28</v>
       </c>
       <c r="G20" s="13">
-        <v>79655.3</v>
+        <v>78324.98</v>
       </c>
       <c r="H20" s="13">
-        <v>16830922.55</v>
+        <v>16600151.86</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -4117,7 +4132,7 @@
         <v>2793591.23</v>
       </c>
       <c r="C21" s="13">
-        <v>234612.6</v>
+        <v>233226.23</v>
       </c>
       <c r="D21" s="13">
         <v>0</v>
@@ -4126,13 +4141,13 @@
         <v>0</v>
       </c>
       <c r="F21" s="13">
-        <v>3028203.83</v>
+        <v>3026817.46</v>
       </c>
       <c r="G21" s="13">
-        <v>98180.38</v>
+        <v>96834.22</v>
       </c>
       <c r="H21" s="13">
-        <v>19957306.76</v>
+        <v>19723803.54</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -4143,7 +4158,7 @@
         <v>2681664.88</v>
       </c>
       <c r="C22" s="13">
-        <v>234612.64</v>
+        <v>233226.27</v>
       </c>
       <c r="D22" s="13">
         <v>0</v>
@@ -4152,13 +4167,13 @@
         <v>0</v>
       </c>
       <c r="F22" s="13">
-        <v>2916277.52</v>
+        <v>2914891.15</v>
       </c>
       <c r="G22" s="13">
-        <v>116417.62</v>
+        <v>115055.52</v>
       </c>
       <c r="H22" s="13">
-        <v>22990001.9</v>
+        <v>22753750.21</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -4169,7 +4184,7 @@
         <v>2527447.05</v>
       </c>
       <c r="C23" s="13">
-        <v>234612.63</v>
+        <v>233226.26</v>
       </c>
       <c r="D23" s="13">
         <v>0</v>
@@ -4178,13 +4193,13 @@
         <v>0</v>
       </c>
       <c r="F23" s="13">
-        <v>2762059.68</v>
+        <v>2760673.31</v>
       </c>
       <c r="G23" s="13">
-        <v>134108.34</v>
+        <v>132730.21</v>
       </c>
       <c r="H23" s="13">
-        <v>25886169.92</v>
+        <v>25647153.73</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -4195,7 +4210,7 @@
         <v>2333369.89</v>
       </c>
       <c r="C24" s="13">
-        <v>234612.59</v>
+        <v>233226.22</v>
       </c>
       <c r="D24" s="13">
         <v>0</v>
@@ -4204,13 +4219,13 @@
         <v>0</v>
       </c>
       <c r="F24" s="13">
-        <v>2567982.48</v>
+        <v>2566596.11</v>
       </c>
       <c r="G24" s="13">
-        <v>151002.66</v>
+        <v>149608.4</v>
       </c>
       <c r="H24" s="13">
-        <v>28605155.06</v>
+        <v>28363358.24</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -4221,7 +4236,7 @@
         <v>2102494.08</v>
       </c>
       <c r="C25" s="13">
-        <v>234612.63</v>
+        <v>233226.26</v>
       </c>
       <c r="D25" s="13">
         <v>0</v>
@@ -4230,13 +4245,13 @@
         <v>0</v>
       </c>
       <c r="F25" s="13">
-        <v>2337106.71</v>
+        <v>2335720.34</v>
       </c>
       <c r="G25" s="13">
-        <v>166863.4</v>
+        <v>165452.92</v>
       </c>
       <c r="H25" s="13">
-        <v>31109125.17</v>
+        <v>30864531.5</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -4247,7 +4262,7 @@
         <v>1838460.71</v>
       </c>
       <c r="C26" s="13">
-        <v>234612.63</v>
+        <v>233226.26</v>
       </c>
       <c r="D26" s="13">
         <v>0</v>
@@ -4256,13 +4271,13 @@
         <v>0</v>
       </c>
       <c r="F26" s="13">
-        <v>2073073.34</v>
+        <v>2071686.97</v>
       </c>
       <c r="G26" s="13">
-        <v>181469.9</v>
+        <v>180043.1</v>
       </c>
       <c r="H26" s="13">
-        <v>33363668.41</v>
+        <v>33116261.57</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -4273,7 +4288,7 @@
         <v>1545433.68</v>
       </c>
       <c r="C27" s="13">
-        <v>234612.59</v>
+        <v>233226.22</v>
       </c>
       <c r="D27" s="13">
         <v>0</v>
@@ -4282,13 +4297,13 @@
         <v>0</v>
       </c>
       <c r="F27" s="13">
-        <v>1780046.27</v>
+        <v>1778659.9</v>
       </c>
       <c r="G27" s="13">
-        <v>194621.4</v>
+        <v>193178.19</v>
       </c>
       <c r="H27" s="13">
-        <v>35338336.08</v>
+        <v>35088099.66</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -4299,7 +4314,7 @@
         <v>1228034.24</v>
       </c>
       <c r="C28" s="13">
-        <v>234612.63</v>
+        <v>233226.26</v>
       </c>
       <c r="D28" s="13">
         <v>0</v>
@@ -4308,13 +4323,13 @@
         <v>0</v>
       </c>
       <c r="F28" s="13">
-        <v>1462646.87</v>
+        <v>1461260.5</v>
       </c>
       <c r="G28" s="13">
-        <v>206140.29</v>
+        <v>204680.58</v>
       </c>
       <c r="H28" s="13">
-        <v>37007123.24</v>
+        <v>36754040.74</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -4325,7 +4340,7 @@
         <v>891267.97</v>
       </c>
       <c r="C29" s="13">
-        <v>234612.62</v>
+        <v>233226.26</v>
       </c>
       <c r="D29" s="13">
         <v>0</v>
@@ -4334,13 +4349,13 @@
         <v>0</v>
       </c>
       <c r="F29" s="13">
-        <v>1125880.59</v>
+        <v>1124494.23</v>
       </c>
       <c r="G29" s="13">
-        <v>215874.89</v>
+        <v>214398.57</v>
       </c>
       <c r="H29" s="13">
-        <v>38348878.72</v>
+        <v>38092933.54</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -4351,7 +4366,7 @@
         <v>540445.9</v>
       </c>
       <c r="C30" s="13">
-        <v>234612.59</v>
+        <v>233226.22</v>
       </c>
       <c r="D30" s="13">
         <v>0</v>
@@ -4360,13 +4375,13 @@
         <v>0</v>
       </c>
       <c r="F30" s="13">
-        <v>775058.49</v>
+        <v>773672.12</v>
       </c>
       <c r="G30" s="13">
-        <v>223701.79</v>
+        <v>222208.78</v>
       </c>
       <c r="H30" s="13">
-        <v>39347639</v>
+        <v>39088814.44</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -4377,7 +4392,7 @@
         <v>181100.68</v>
       </c>
       <c r="C31" s="13">
-        <v>234612.62</v>
+        <v>233226.26</v>
       </c>
       <c r="D31" s="13">
         <v>0</v>
@@ -4386,13 +4401,13 @@
         <v>0</v>
       </c>
       <c r="F31" s="13">
-        <v>415713.3</v>
+        <v>414326.94</v>
       </c>
       <c r="G31" s="13">
-        <v>229527.89</v>
+        <v>228018.08</v>
       </c>
       <c r="H31" s="13">
-        <v>39992880.19</v>
+        <v>39731159.46</v>
       </c>
     </row>
   </sheetData>
@@ -4414,7 +4429,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -5419,6 +5434,26 @@
       </c>
       <c r="F56" s="12" t="s">
         <v>336</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="B57" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="F57" s="12" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>